<commit_message>
Freeze headers only on the long scrollable lists
Re-enable frozen column headers on the three tabs where scrolling past the
header actually happens (Wedding Checklist, Guest List, Gifts and Thank You)
so the headers stay visible. All other tabs stay unfrozen, so the freeze-pane
divider line only appears where it earns its place.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LBuV472FujAVwRm4KPoq6q
</commit_message>
<xml_diff>
--- a/dist/Wedding-Planner-All-In-One.xlsx
+++ b/dist/Wedding-Planner-All-In-One.xlsx
@@ -6819,11 +6819,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="98346222"/>
-        <c:axId val="95598873"/>
+        <c:axId val="72130385"/>
+        <c:axId val="18722873"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="98346222"/>
+        <c:axId val="72130385"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6855,7 +6855,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="95598873"/>
+        <c:crossAx val="18722873"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -6863,7 +6863,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="95598873"/>
+        <c:axId val="18722873"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6895,7 +6895,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="98346222"/>
+        <c:crossAx val="72130385"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -7582,11 +7582,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="54052013"/>
-        <c:axId val="6349449"/>
+        <c:axId val="39179791"/>
+        <c:axId val="94226096"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="54052013"/>
+        <c:axId val="39179791"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7618,7 +7618,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="6349449"/>
+        <c:crossAx val="94226096"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -7626,7 +7626,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="6349449"/>
+        <c:axId val="94226096"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7658,7 +7658,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="54052013"/>
+        <c:crossAx val="39179791"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -7830,11 +7830,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="55515679"/>
-        <c:axId val="79331679"/>
+        <c:axId val="80024276"/>
+        <c:axId val="50846560"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="55515679"/>
+        <c:axId val="80024276"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7866,7 +7866,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="79331679"/>
+        <c:crossAx val="50846560"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -7874,7 +7874,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="79331679"/>
+        <c:axId val="50846560"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7906,7 +7906,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="55515679"/>
+        <c:crossAx val="80024276"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -8096,11 +8096,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="36518614"/>
-        <c:axId val="25591665"/>
+        <c:axId val="95051354"/>
+        <c:axId val="18957805"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="36518614"/>
+        <c:axId val="95051354"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8132,7 +8132,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="25591665"/>
+        <c:crossAx val="18957805"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -8140,7 +8140,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="25591665"/>
+        <c:axId val="18957805"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8172,7 +8172,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="36518614"/>
+        <c:crossAx val="95051354"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -8356,11 +8356,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="71393992"/>
-        <c:axId val="36504421"/>
+        <c:axId val="24199499"/>
+        <c:axId val="94282676"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="71393992"/>
+        <c:axId val="24199499"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8392,7 +8392,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="36504421"/>
+        <c:crossAx val="94282676"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -8400,7 +8400,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="36504421"/>
+        <c:axId val="94282676"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8432,7 +8432,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="71393992"/>
+        <c:crossAx val="24199499"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -8586,11 +8586,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="94526433"/>
-        <c:axId val="6871880"/>
+        <c:axId val="49601498"/>
+        <c:axId val="31837570"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="94526433"/>
+        <c:axId val="49601498"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8622,7 +8622,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="6871880"/>
+        <c:crossAx val="31837570"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -8630,7 +8630,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="6871880"/>
+        <c:axId val="31837570"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8662,7 +8662,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="94526433"/>
+        <c:crossAx val="49601498"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -8822,11 +8822,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="50024369"/>
-        <c:axId val="56978632"/>
+        <c:axId val="14675865"/>
+        <c:axId val="87810862"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="50024369"/>
+        <c:axId val="14675865"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8858,7 +8858,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="56978632"/>
+        <c:crossAx val="87810862"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -8866,7 +8866,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="56978632"/>
+        <c:axId val="87810862"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8898,7 +8898,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="50024369"/>
+        <c:crossAx val="14675865"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -11375,11 +11375,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="36592648"/>
-        <c:axId val="31244834"/>
+        <c:axId val="86993302"/>
+        <c:axId val="41499633"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="36592648"/>
+        <c:axId val="86993302"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -11411,7 +11411,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="31244834"/>
+        <c:crossAx val="41499633"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -11419,7 +11419,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="31244834"/>
+        <c:axId val="41499633"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -11451,7 +11451,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="36592648"/>
+        <c:crossAx val="86993302"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -11866,11 +11866,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="75201424"/>
-        <c:axId val="44236749"/>
+        <c:axId val="67305794"/>
+        <c:axId val="60145589"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="75201424"/>
+        <c:axId val="67305794"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -11902,7 +11902,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="44236749"/>
+        <c:crossAx val="60145589"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -11910,7 +11910,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="44236749"/>
+        <c:axId val="60145589"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -11942,7 +11942,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="75201424"/>
+        <c:crossAx val="67305794"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -12474,11 +12474,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="68003451"/>
-        <c:axId val="44454610"/>
+        <c:axId val="61555467"/>
+        <c:axId val="80119946"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="68003451"/>
+        <c:axId val="61555467"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -12510,7 +12510,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="44454610"/>
+        <c:crossAx val="80119946"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -12518,7 +12518,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="44454610"/>
+        <c:axId val="80119946"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -12550,7 +12550,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="68003451"/>
+        <c:crossAx val="61555467"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -12898,11 +12898,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="86859151"/>
-        <c:axId val="37287007"/>
+        <c:axId val="4239967"/>
+        <c:axId val="4923004"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="86859151"/>
+        <c:axId val="4239967"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -12934,7 +12934,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="37287007"/>
+        <c:crossAx val="4923004"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -12942,7 +12942,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="37287007"/>
+        <c:axId val="4923004"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -12974,7 +12974,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="86859151"/>
+        <c:crossAx val="4239967"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -13206,11 +13206,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="74801723"/>
-        <c:axId val="38012479"/>
+        <c:axId val="99395440"/>
+        <c:axId val="72770285"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="74801723"/>
+        <c:axId val="99395440"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -13242,7 +13242,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="38012479"/>
+        <c:crossAx val="72770285"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -13250,7 +13250,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="38012479"/>
+        <c:axId val="72770285"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -13282,7 +13282,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="74801723"/>
+        <c:crossAx val="99395440"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -14159,11 +14159,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="5375510"/>
-        <c:axId val="35382992"/>
+        <c:axId val="44891372"/>
+        <c:axId val="7335932"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="5375510"/>
+        <c:axId val="44891372"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -14195,7 +14195,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="35382992"/>
+        <c:crossAx val="7335932"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -14203,7 +14203,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="35382992"/>
+        <c:axId val="7335932"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -14235,7 +14235,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="5375510"/>
+        <c:crossAx val="44891372"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>

<commit_message>
Freeze headers on all single-table tabs
Enable frozen column headers on every tab that has one main scrollable table
(20 tabs), including Decor, Flowers and Stationery. Tabs with no single header
row (multi-section party/logistics/music tabs) or no table at all (Dashboard,
Get Started, Calendar, Moodboard, Save the Date) are left unfrozen.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LBuV472FujAVwRm4KPoq6q
</commit_message>
<xml_diff>
--- a/dist/Wedding-Planner-All-In-One.xlsx
+++ b/dist/Wedding-Planner-All-In-One.xlsx
@@ -6819,11 +6819,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="72130385"/>
-        <c:axId val="18722873"/>
+        <c:axId val="82956033"/>
+        <c:axId val="57581551"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="72130385"/>
+        <c:axId val="82956033"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6855,7 +6855,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="18722873"/>
+        <c:crossAx val="57581551"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -6863,7 +6863,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="18722873"/>
+        <c:axId val="57581551"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6895,7 +6895,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="72130385"/>
+        <c:crossAx val="82956033"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -7582,11 +7582,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="39179791"/>
-        <c:axId val="94226096"/>
+        <c:axId val="66318600"/>
+        <c:axId val="88783639"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="39179791"/>
+        <c:axId val="66318600"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7618,7 +7618,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="94226096"/>
+        <c:crossAx val="88783639"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -7626,7 +7626,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="94226096"/>
+        <c:axId val="88783639"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7658,7 +7658,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="39179791"/>
+        <c:crossAx val="66318600"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -7830,11 +7830,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="80024276"/>
-        <c:axId val="50846560"/>
+        <c:axId val="60487119"/>
+        <c:axId val="46071228"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="80024276"/>
+        <c:axId val="60487119"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7866,7 +7866,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="50846560"/>
+        <c:crossAx val="46071228"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -7874,7 +7874,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="50846560"/>
+        <c:axId val="46071228"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7906,7 +7906,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="80024276"/>
+        <c:crossAx val="60487119"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -8096,11 +8096,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="95051354"/>
-        <c:axId val="18957805"/>
+        <c:axId val="71686446"/>
+        <c:axId val="80485631"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="95051354"/>
+        <c:axId val="71686446"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8132,7 +8132,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="18957805"/>
+        <c:crossAx val="80485631"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -8140,7 +8140,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="18957805"/>
+        <c:axId val="80485631"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8172,7 +8172,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="95051354"/>
+        <c:crossAx val="71686446"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -8356,11 +8356,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="24199499"/>
-        <c:axId val="94282676"/>
+        <c:axId val="9282771"/>
+        <c:axId val="37164128"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="24199499"/>
+        <c:axId val="9282771"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8392,7 +8392,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="94282676"/>
+        <c:crossAx val="37164128"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -8400,7 +8400,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="94282676"/>
+        <c:axId val="37164128"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8432,7 +8432,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="24199499"/>
+        <c:crossAx val="9282771"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -8586,11 +8586,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="49601498"/>
-        <c:axId val="31837570"/>
+        <c:axId val="91602965"/>
+        <c:axId val="84366139"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="49601498"/>
+        <c:axId val="91602965"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8622,7 +8622,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="31837570"/>
+        <c:crossAx val="84366139"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -8630,7 +8630,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="31837570"/>
+        <c:axId val="84366139"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8662,7 +8662,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="49601498"/>
+        <c:crossAx val="91602965"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -8822,11 +8822,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="14675865"/>
-        <c:axId val="87810862"/>
+        <c:axId val="59003655"/>
+        <c:axId val="25491521"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="14675865"/>
+        <c:axId val="59003655"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8858,7 +8858,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="87810862"/>
+        <c:crossAx val="25491521"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -8866,7 +8866,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="87810862"/>
+        <c:axId val="25491521"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8898,7 +8898,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="14675865"/>
+        <c:crossAx val="59003655"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -11375,11 +11375,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="86993302"/>
-        <c:axId val="41499633"/>
+        <c:axId val="32516083"/>
+        <c:axId val="42938501"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="86993302"/>
+        <c:axId val="32516083"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -11411,7 +11411,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="41499633"/>
+        <c:crossAx val="42938501"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -11419,7 +11419,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="41499633"/>
+        <c:axId val="42938501"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -11451,7 +11451,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="86993302"/>
+        <c:crossAx val="32516083"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -11866,11 +11866,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="67305794"/>
-        <c:axId val="60145589"/>
+        <c:axId val="33366213"/>
+        <c:axId val="7906641"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="67305794"/>
+        <c:axId val="33366213"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -11902,7 +11902,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="60145589"/>
+        <c:crossAx val="7906641"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -11910,7 +11910,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="60145589"/>
+        <c:axId val="7906641"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -11942,7 +11942,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="67305794"/>
+        <c:crossAx val="33366213"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -12474,11 +12474,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="61555467"/>
-        <c:axId val="80119946"/>
+        <c:axId val="9374041"/>
+        <c:axId val="94208852"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="61555467"/>
+        <c:axId val="9374041"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -12510,7 +12510,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="80119946"/>
+        <c:crossAx val="94208852"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -12518,7 +12518,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="80119946"/>
+        <c:axId val="94208852"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -12550,7 +12550,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="61555467"/>
+        <c:crossAx val="9374041"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -12898,11 +12898,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="4239967"/>
-        <c:axId val="4923004"/>
+        <c:axId val="25309719"/>
+        <c:axId val="30541203"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="4239967"/>
+        <c:axId val="25309719"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -12934,7 +12934,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="4923004"/>
+        <c:crossAx val="30541203"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -12942,7 +12942,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="4923004"/>
+        <c:axId val="30541203"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -12974,7 +12974,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="4239967"/>
+        <c:crossAx val="25309719"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -13206,11 +13206,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="99395440"/>
-        <c:axId val="72770285"/>
+        <c:axId val="18936560"/>
+        <c:axId val="49144451"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="99395440"/>
+        <c:axId val="18936560"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -13242,7 +13242,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="72770285"/>
+        <c:crossAx val="49144451"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -13250,7 +13250,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="72770285"/>
+        <c:axId val="49144451"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -13282,7 +13282,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="99395440"/>
+        <c:crossAx val="18936560"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -14159,11 +14159,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="44891372"/>
-        <c:axId val="7335932"/>
+        <c:axId val="50772334"/>
+        <c:axId val="12516956"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="44891372"/>
+        <c:axId val="50772334"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -14195,7 +14195,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="7335932"/>
+        <c:crossAx val="12516956"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -14203,7 +14203,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="7335932"/>
+        <c:axId val="12516956"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -14235,7 +14235,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="44891372"/>
+        <c:crossAx val="50772334"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>